<commit_message>
fix: adiciona inst/WORDLIST para corrigir verificação ortográfica do CRAN
</commit_message>
<xml_diff>
--- a/inst/extdata/executado.xlsx
+++ b/inst/extdata/executado.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/54ecef3130cc9632/Área de Trabalho/mifebpc/inst/extdata/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hernany.castro\Desktop\orcamento\mifebpc\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{2EE580D0-2853-4787-9AB3-89A44900FB65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F657B644-8CE9-45B8-8286-A56BCBBA20A5}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B12012A1-9134-46E1-BC78-67C1DB19D432}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="resumo_financeiro" sheetId="6" r:id="rId1"/>
@@ -116,7 +116,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -132,7 +132,6 @@
     <xf numFmtId="17" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -471,7 +470,7 @@
         <v>4344731582.1800003</v>
       </c>
       <c r="D2" s="4">
-        <f>B2+C2</f>
+        <f t="shared" ref="D2:D9" si="0">B2+C2</f>
         <v>10584658239.799999</v>
       </c>
     </row>
@@ -486,7 +485,7 @@
         <v>4443307320.0100002</v>
       </c>
       <c r="D3" s="4">
-        <f>B3+C3</f>
+        <f t="shared" si="0"/>
         <v>10766881908.67</v>
       </c>
     </row>
@@ -501,7 +500,7 @@
         <v>4772276369.9200001</v>
       </c>
       <c r="D4" s="4">
-        <f>B4+C4</f>
+        <f t="shared" si="0"/>
         <v>11385397540.42</v>
       </c>
     </row>
@@ -516,7 +515,7 @@
         <v>4524961581.7399998</v>
       </c>
       <c r="D5" s="4">
-        <f>B5+C5</f>
+        <f t="shared" si="0"/>
         <v>11024401537.48</v>
       </c>
     </row>
@@ -531,7 +530,7 @@
         <v>4444390885.1899996</v>
       </c>
       <c r="D6" s="4">
-        <f>B6+C6</f>
+        <f t="shared" si="0"/>
         <v>10851476138.48</v>
       </c>
     </row>
@@ -546,7 +545,7 @@
         <v>4537836366.9700003</v>
       </c>
       <c r="D7" s="4">
-        <f>B7+C7</f>
+        <f t="shared" si="0"/>
         <v>11019011283.060001</v>
       </c>
     </row>
@@ -561,7 +560,7 @@
         <v>4686335425.1499996</v>
       </c>
       <c r="D8" s="4">
-        <f>B8+C8</f>
+        <f t="shared" si="0"/>
         <v>11387636241.689999</v>
       </c>
     </row>
@@ -576,27 +575,37 @@
         <v>4420909574.7600002</v>
       </c>
       <c r="D9" s="4">
-        <f>B9+C9</f>
+        <f t="shared" si="0"/>
         <v>10657448647.82</v>
       </c>
-      <c r="E9" s="10"/>
+      <c r="E9" s="9"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="7"/>
+      <c r="A10" s="6">
+        <v>46266</v>
+      </c>
+      <c r="B10" s="3">
+        <v>6585442622.1300001</v>
+      </c>
+      <c r="C10" s="3">
+        <v>4586527855.4300003</v>
+      </c>
+      <c r="D10" s="4">
+        <f t="shared" ref="D10" si="1">B10+C10</f>
+        <v>11171970477.560001</v>
+      </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B11" s="1"/>
-      <c r="D11" s="8"/>
+      <c r="D11" s="7"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B13" s="9"/>
-      <c r="C13" s="9"/>
+      <c r="B13" s="8"/>
+      <c r="C13" s="8"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C15" s="1"/>

</xml_diff>